<commit_message>
Sskx: Update filling column N (#2633)
* Sskz: Update filling column N

* update sskx excel template

* Update table reference

* Remove temporary file

* update xsl reference

---------

Co-authored-by: eclipse-set-bot <set-bot@eclipse.org>
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SET\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755332A6-D571-492E-9FFC-FA418024C307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B2B844-9C61-4E00-BCE0-4891DBEC6A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="12645" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskx_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
   <si>
     <t>A</t>
   </si>
@@ -145,18 +145,19 @@
 Rz. Nr. (Bild)</t>
   </si>
   <si>
-    <t>Signalbegriff</t>
-  </si>
-  <si>
     <t>Gleis</t>
-  </si>
-  <si>
-    <t>Bezeichnung (Symbol)</t>
   </si>
   <si>
     <t>Abstand/Lage
 Mastmitte - Gleismitte
 (Gleisabstand)</t>
+  </si>
+  <si>
+    <t>Weitere Regelzeichnung
+Nr. (Bild)</t>
+  </si>
+  <si>
+    <t>Signalbegriff Bezeichnung (Symbol)</t>
   </si>
 </sst>
 </file>
@@ -199,7 +200,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -441,6 +442,19 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -448,7 +462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -562,6 +576,18 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1049,7 +1075,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="31" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I3" s="32"/>
       <c r="J3" s="33" t="s">
@@ -1060,13 +1086,15 @@
         <v>23</v>
       </c>
       <c r="M3" s="34"/>
-      <c r="N3" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="O3" s="34"/>
+      <c r="N3" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" s="40" t="s">
+        <v>36</v>
+      </c>
       <c r="P3" s="20"/>
     </row>
-    <row r="4" spans="1:16" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5" t="s">
@@ -1076,7 +1104,7 @@
         <v>25</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -1098,15 +1126,11 @@
       <c r="M4" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>27</v>
-      </c>
+      <c r="N4" s="39"/>
+      <c r="O4" s="41"/>
       <c r="P4" s="16"/>
     </row>
-    <row r="5" spans="1:16" s="2" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" s="2" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="9"/>
       <c r="C5" s="10"/>
@@ -1683,15 +1707,16 @@
       <c r="P55" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="H3:I3"/>
-    <mergeCell ref="N3:O3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="L3:M3"/>
     <mergeCell ref="J2:M2"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>

</xml_diff>